<commit_message>
Revisão do parecer: versão final após segunda verificação (notas na ordem, normalização de PC e TN, contrafactual)
Renumera as notas na ordem das chamadas (o LibreOffice exibia textos trocados),
registra que PC e TN foram divididos pelo máximo na planilha, mede o PCM como
descrito no texto (rho 0,99; 153 de 157 seleções), explicita que os ajustes de
maio passaram à frente de suplentes com PCM maior, informa a versão de março e
o contrafactual com a etapa prévia fixa (152 municípios), marca os argumentos
técnicos dos pesos como verificação a posteriori e corrige a versão com marcas
(trechos duplicados). Atualiza planilha de dados, suplementares, carta e a
auditoria (variante da faixa P3 também na planilha de maio).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MDzyNreLrve5brDgfNKZ3e
</commit_message>
<xml_diff>
--- a/creches-parana/10_revisao_parecer/Material_Suplementar/Tabelas_1_a_7_dados_editaveis.xlsx
+++ b/creches-parana/10_revisao_parecer/Material_Suplementar/Tabelas_1_a_7_dados_editaveis.xlsx
@@ -1609,7 +1609,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Mun/</t>
+          <t>Mun.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>100 após tetos</t>
+          <t>100 (cota fixa)</t>
         </is>
       </c>
     </row>

</xml_diff>